<commit_message>
big phrazer update 2021_04
</commit_message>
<xml_diff>
--- a/_appdata/_extern/Wartezeiten Modell 2 (LengthBased) Shorter.xlsx
+++ b/_appdata/_extern/Wartezeiten Modell 2 (LengthBased) Shorter.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>thinkingTime</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>signs</t>
+  </si>
+  <si>
+    <t>2 REPEATS</t>
   </si>
 </sst>
 </file>
@@ -94,7 +97,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -116,6 +119,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -141,12 +150,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -427,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="D2:N24"/>
+  <dimension ref="A2:O27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="15.42578125" customWidth="1"/>
@@ -438,22 +447,22 @@
     <col min="12" max="14" width="7.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="4:14" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="D2" s="9" t="s">
+    <row r="2" spans="1:14" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="D2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="K2" s="9" t="s">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="K2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-    </row>
-    <row r="3" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
         <v>10</v>
       </c>
@@ -482,25 +491,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="4:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D5" s="2">
         <v>10</v>
       </c>
       <c r="E5" s="2">
-        <f>D5*0.005+1</f>
+        <f t="shared" ref="E5:E19" si="0">D5*0.005+1</f>
         <v>1.05</v>
       </c>
       <c r="F5" s="2">
-        <f>D5*0.08+1.5</f>
-        <v>2.2999999999999998</v>
+        <f>D5*0.05+2</f>
+        <v>2.5</v>
       </c>
       <c r="G5" s="2">
         <f>E5+F5</f>
-        <v>3.3499999999999996</v>
+        <v>3.55</v>
       </c>
       <c r="H5" s="2">
         <f>F5</f>
-        <v>2.2999999999999998</v>
+        <v>2.5</v>
       </c>
       <c r="K5" s="2">
         <v>0.25</v>
@@ -515,25 +524,25 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="6" spans="4:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D6" s="4">
         <v>20</v>
       </c>
       <c r="E6" s="2">
-        <f t="shared" ref="E6:E24" si="0">D6*0.005+1</f>
+        <f t="shared" si="0"/>
         <v>1.1000000000000001</v>
       </c>
       <c r="F6" s="2">
-        <f t="shared" ref="F6:F24" si="1">D6*0.08+1.5</f>
-        <v>3.1</v>
+        <f t="shared" ref="F6:F13" si="1">D6*0.05+2</f>
+        <v>3</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:G24" si="2">E6+F6</f>
-        <v>4.2</v>
+        <f t="shared" ref="G6:G19" si="2">E6+F6</f>
+        <v>4.0999999999999996</v>
       </c>
       <c r="H6">
-        <f t="shared" ref="H6:H24" si="3">F6</f>
-        <v>3.1</v>
+        <f t="shared" ref="H6:H19" si="3">F6</f>
+        <v>3</v>
       </c>
       <c r="M6">
         <v>3</v>
@@ -542,7 +551,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="7" spans="4:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D7" s="5">
         <v>30</v>
       </c>
@@ -552,18 +561,18 @@
       </c>
       <c r="F7" s="2">
         <f t="shared" si="1"/>
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="G7">
         <f t="shared" si="2"/>
-        <v>5.05</v>
+        <v>4.6500000000000004</v>
       </c>
       <c r="H7">
         <f t="shared" si="3"/>
-        <v>3.9</v>
-      </c>
-    </row>
-    <row r="8" spans="4:14" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D8" s="4">
         <v>40</v>
       </c>
@@ -573,18 +582,18 @@
       </c>
       <c r="F8" s="2">
         <f t="shared" si="1"/>
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="G8">
         <f t="shared" si="2"/>
-        <v>5.9</v>
+        <v>5.2</v>
       </c>
       <c r="H8">
         <f t="shared" si="3"/>
-        <v>4.7</v>
-      </c>
-    </row>
-    <row r="9" spans="4:14" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D9" s="5">
         <v>50</v>
       </c>
@@ -594,18 +603,18 @@
       </c>
       <c r="F9" s="2">
         <f t="shared" si="1"/>
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="G9">
         <f t="shared" si="2"/>
-        <v>6.75</v>
+        <v>5.75</v>
       </c>
       <c r="H9">
         <f t="shared" si="3"/>
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="10" spans="4:14" x14ac:dyDescent="0.25">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D10" s="4">
         <v>60</v>
       </c>
@@ -615,18 +624,18 @@
       </c>
       <c r="F10" s="2">
         <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="2"/>
         <v>6.3</v>
       </c>
-      <c r="G10">
-        <f t="shared" si="2"/>
-        <v>7.6</v>
-      </c>
       <c r="H10">
         <f t="shared" si="3"/>
-        <v>6.3</v>
-      </c>
-    </row>
-    <row r="11" spans="4:14" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D11" s="5">
         <v>70</v>
       </c>
@@ -636,301 +645,293 @@
       </c>
       <c r="F11" s="2">
         <f t="shared" si="1"/>
-        <v>7.1000000000000005</v>
+        <v>5.5</v>
       </c>
       <c r="G11">
         <f t="shared" si="2"/>
-        <v>8.4500000000000011</v>
+        <v>6.85</v>
       </c>
       <c r="H11">
         <f t="shared" si="3"/>
-        <v>7.1000000000000005</v>
-      </c>
-    </row>
-    <row r="12" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D12" s="4">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="9">
         <v>80</v>
       </c>
       <c r="E12" s="2">
-        <f t="shared" si="0"/>
-        <v>1.4</v>
+        <v>-1</v>
       </c>
       <c r="F12" s="2">
-        <f t="shared" si="1"/>
-        <v>7.9</v>
-      </c>
-      <c r="G12">
-        <f t="shared" si="2"/>
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="H12">
-        <f t="shared" si="3"/>
-        <v>7.9</v>
-      </c>
-    </row>
-    <row r="13" spans="4:14" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="G12" s="9">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="H12" s="9">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D13" s="5">
         <v>90</v>
       </c>
       <c r="E13" s="2">
-        <f t="shared" si="0"/>
-        <v>1.45</v>
+        <v>-1</v>
       </c>
       <c r="F13" s="2">
-        <f t="shared" si="1"/>
-        <v>8.6999999999999993</v>
+        <v>4</v>
       </c>
       <c r="G13">
         <f t="shared" si="2"/>
-        <v>10.149999999999999</v>
+        <v>3</v>
       </c>
       <c r="H13">
         <f t="shared" si="3"/>
-        <v>8.6999999999999993</v>
-      </c>
-    </row>
-    <row r="14" spans="4:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D14" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D14" s="4">
         <v>100</v>
       </c>
       <c r="E14" s="2">
-        <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>-1</v>
       </c>
       <c r="F14" s="2">
-        <f t="shared" si="1"/>
-        <v>9.5</v>
-      </c>
-      <c r="G14" s="2">
-        <f t="shared" si="2"/>
-        <v>11</v>
-      </c>
-      <c r="H14" s="2">
-        <f t="shared" si="3"/>
-        <v>9.5</v>
-      </c>
-      <c r="K14" s="2">
+        <v>4</v>
+      </c>
+      <c r="G14" s="5">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="H14" s="5">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="K14" s="5">
         <v>2</v>
       </c>
-      <c r="L14" s="2">
+      <c r="L14" s="5">
         <v>5</v>
       </c>
-      <c r="M14" s="2">
+      <c r="M14" s="5">
         <v>7</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="5">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="4:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D15" s="5">
         <v>110</v>
       </c>
       <c r="E15" s="2">
-        <f t="shared" si="0"/>
-        <v>1.55</v>
+        <v>-1</v>
       </c>
       <c r="F15" s="2">
-        <f t="shared" si="1"/>
-        <v>10.3</v>
+        <v>4</v>
       </c>
       <c r="G15">
         <f t="shared" si="2"/>
-        <v>11.850000000000001</v>
+        <v>3</v>
       </c>
       <c r="H15">
         <f t="shared" si="3"/>
-        <v>10.3</v>
-      </c>
-    </row>
-    <row r="16" spans="4:14" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D16" s="4">
         <v>120</v>
       </c>
       <c r="E16" s="2">
-        <f t="shared" si="0"/>
-        <v>1.6</v>
+        <v>-1</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" si="1"/>
-        <v>11.1</v>
+        <v>4</v>
       </c>
       <c r="G16">
         <f t="shared" si="2"/>
-        <v>12.7</v>
+        <v>3</v>
       </c>
       <c r="H16">
         <f t="shared" si="3"/>
-        <v>11.1</v>
-      </c>
-    </row>
-    <row r="17" spans="4:8" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D17" s="5">
         <v>130</v>
       </c>
       <c r="E17" s="2">
-        <f t="shared" si="0"/>
-        <v>1.65</v>
+        <v>-1</v>
       </c>
       <c r="F17" s="2">
-        <f t="shared" si="1"/>
-        <v>11.9</v>
+        <v>4</v>
       </c>
       <c r="G17">
         <f t="shared" si="2"/>
-        <v>13.55</v>
+        <v>3</v>
       </c>
       <c r="H17">
         <f t="shared" si="3"/>
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="18" spans="4:8" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D18" s="4">
         <v>140</v>
       </c>
       <c r="E18" s="2">
-        <f t="shared" si="0"/>
-        <v>1.7000000000000002</v>
+        <v>-1</v>
       </c>
       <c r="F18" s="2">
-        <f t="shared" si="1"/>
-        <v>12.700000000000001</v>
-      </c>
-      <c r="G18">
-        <f t="shared" si="2"/>
-        <v>14.400000000000002</v>
-      </c>
-      <c r="H18">
-        <f t="shared" si="3"/>
-        <v>12.700000000000001</v>
-      </c>
-    </row>
-    <row r="19" spans="4:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="7">
+        <v>4</v>
+      </c>
+      <c r="G18" s="4">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="H18" s="4">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+    </row>
+    <row r="19" spans="1:15" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D19" s="6">
         <v>150</v>
       </c>
       <c r="E19" s="2">
-        <f t="shared" si="0"/>
-        <v>1.75</v>
+        <v>-1</v>
       </c>
       <c r="F19" s="2">
-        <f t="shared" si="1"/>
-        <v>13.5</v>
-      </c>
-      <c r="G19" s="8">
-        <f t="shared" si="2"/>
-        <v>15.25</v>
-      </c>
-      <c r="H19" s="8">
-        <f t="shared" si="3"/>
-        <v>13.5</v>
-      </c>
-    </row>
-    <row r="20" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D20" s="4">
-        <v>160</v>
-      </c>
-      <c r="E20" s="2">
-        <f t="shared" si="0"/>
-        <v>1.8</v>
-      </c>
-      <c r="F20" s="2">
-        <f t="shared" si="1"/>
-        <v>14.3</v>
-      </c>
-      <c r="G20">
-        <f t="shared" si="2"/>
-        <v>16.100000000000001</v>
-      </c>
-      <c r="H20">
-        <f t="shared" si="3"/>
-        <v>14.3</v>
-      </c>
-    </row>
-    <row r="21" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D21" s="5">
-        <v>170</v>
-      </c>
-      <c r="E21" s="2">
-        <f t="shared" si="0"/>
-        <v>1.85</v>
-      </c>
-      <c r="F21" s="2">
-        <f t="shared" si="1"/>
-        <v>15.1</v>
-      </c>
-      <c r="G21">
-        <f t="shared" si="2"/>
-        <v>16.95</v>
-      </c>
-      <c r="H21">
-        <f t="shared" si="3"/>
-        <v>15.1</v>
-      </c>
-    </row>
-    <row r="22" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D22" s="4">
-        <v>180</v>
-      </c>
-      <c r="E22" s="2">
-        <f t="shared" si="0"/>
-        <v>1.9</v>
-      </c>
-      <c r="F22" s="2">
-        <f t="shared" si="1"/>
-        <v>15.9</v>
-      </c>
-      <c r="G22">
-        <f t="shared" si="2"/>
-        <v>17.8</v>
-      </c>
-      <c r="H22">
-        <f t="shared" si="3"/>
-        <v>15.9</v>
-      </c>
-    </row>
-    <row r="23" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D23" s="5">
-        <v>190</v>
-      </c>
-      <c r="E23" s="2">
-        <f t="shared" si="0"/>
-        <v>1.9500000000000002</v>
-      </c>
-      <c r="F23" s="2">
-        <f t="shared" si="1"/>
-        <v>16.700000000000003</v>
-      </c>
-      <c r="G23">
-        <f t="shared" si="2"/>
-        <v>18.650000000000002</v>
-      </c>
-      <c r="H23">
-        <f t="shared" si="3"/>
-        <v>16.700000000000003</v>
-      </c>
-    </row>
-    <row r="24" spans="4:8" x14ac:dyDescent="0.25">
-      <c r="D24" s="4">
-        <v>200</v>
-      </c>
-      <c r="E24" s="2">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="F24" s="2">
-        <f t="shared" si="1"/>
-        <v>17.5</v>
-      </c>
-      <c r="G24">
-        <f t="shared" si="2"/>
-        <v>19.5</v>
-      </c>
-      <c r="H24">
-        <f t="shared" si="3"/>
-        <v>17.5</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G19" s="4">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="H19" s="4">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D21" s="4"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>